<commit_message>
Update experiment_statistics: drop queueing-formula row, keep table only
</commit_message>
<xml_diff>
--- a/experiment_statistics.xlsx
+++ b/experiment_statistics.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,11 +35,6 @@
     <font>
       <name val="Calibri"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <sz val="10"/>
     </font>
   </fonts>
   <fills count="2">
@@ -76,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -90,7 +85,6 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -456,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -490,72 +484,49 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Queueing formula</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>15.28</v>
+        <v>18.39</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>17.1</v>
+        <v>36.64</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>0.9992</v>
+        <v>0.9964</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>Linear Regression</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>18.39</v>
+        <v>271.72</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>36.64</v>
+        <v>431.47</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>0.9964</v>
+        <v>0.5018</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Linear Regression</t>
+          <t>Dummy Regressor</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>271.72</v>
+        <v>306.69</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>431.47</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>0.5018</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Dummy Regressor</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>306.69</v>
-      </c>
-      <c r="C5" s="3" t="n">
         <v>646.3</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D4" s="3" t="n">
         <v>-0.12</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Note: lower MAE/RMSE is better; higher R2 is generally better (1.0 = perfect).</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>